<commit_message>
Refine Q2 routes and shared-battery schedules
# Conflicts:
#	README.md
</commit_message>
<xml_diff>
--- a/results_q2/q2_result_template.xlsx
+++ b/results_q2/q2_result_template.xlsx
@@ -1303,7 +1303,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H29"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="2"/>
   <cols>
     <col width="12" customWidth="1" style="3" min="1" max="2"/>
@@ -1384,14 +1384,14 @@
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>S006→S007</t>
+          <t>S002</t>
         </is>
       </c>
       <c r="G2" s="4" t="n">
-        <v>2404.597883</v>
+        <v>2115.081641</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>4.285813</v>
+        <v>6.126766</v>
       </c>
     </row>
     <row r="3">
@@ -1438,32 +1438,32 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>U08</t>
+          <t>U05</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>C03</t>
+          <t>B01</t>
         </is>
       </c>
       <c r="E4" s="4" t="n">
-        <v>1495.426178</v>
+        <v>0</v>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>S002</t>
+          <t>S010</t>
         </is>
       </c>
       <c r="G4" s="4" t="n">
-        <v>3610.507819</v>
+        <v>1554.571359</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>6.126766</v>
+        <v>1.821045</v>
       </c>
     </row>
     <row r="5">
@@ -1474,7 +1474,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>U05</t>
+          <t>U06</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
@@ -1484,7 +1484,7 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>B01</t>
+          <t>B02</t>
         </is>
       </c>
       <c r="E5" s="4" t="n">
@@ -1492,14 +1492,14 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>S006</t>
+          <t>S013</t>
         </is>
       </c>
       <c r="G5" s="4" t="n">
-        <v>1209.979917</v>
+        <v>1440.969393</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>1.098424</v>
+        <v>1.632661</v>
       </c>
     </row>
     <row r="6">
@@ -1510,17 +1510,17 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>U06</t>
+          <t>U01</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>B02</t>
+          <t>A01</t>
         </is>
       </c>
       <c r="E6" s="4" t="n">
@@ -1528,14 +1528,14 @@
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>S013</t>
+          <t>S001</t>
         </is>
       </c>
       <c r="G6" s="4" t="n">
-        <v>1440.969393</v>
+        <v>1312.470877</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>1.632661</v>
+        <v>1.268023</v>
       </c>
     </row>
     <row r="7">
@@ -1546,32 +1546,32 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>U07</t>
+          <t>U02</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>C04</t>
+          <t>A02</t>
         </is>
       </c>
       <c r="E7" s="4" t="n">
-        <v>2404.597883</v>
+        <v>0</v>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>S001</t>
+          <t>S011</t>
         </is>
       </c>
       <c r="G7" s="4" t="n">
-        <v>3900.02406</v>
+        <v>1223.535214</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>2.672703</v>
+        <v>1.15549</v>
       </c>
     </row>
     <row r="8">
@@ -1592,22 +1592,22 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>C02</t>
+          <t>C03</t>
         </is>
       </c>
       <c r="E8" s="4" t="n">
-        <v>3610.507819</v>
+        <v>1495.426178</v>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>S003</t>
+          <t>S006→S007</t>
         </is>
       </c>
       <c r="G8" s="4" t="n">
-        <v>6046.31734</v>
+        <v>3966.02406</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>6.14777</v>
+        <v>4.569801</v>
       </c>
     </row>
     <row r="9">
@@ -1618,32 +1618,32 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>U05</t>
+          <t>U03</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>B03</t>
+          <t>A03</t>
         </is>
       </c>
       <c r="E9" s="4" t="n">
-        <v>1209.979917</v>
+        <v>0</v>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>S010→S014</t>
+          <t>S009→S002</t>
         </is>
       </c>
       <c r="G9" s="4" t="n">
-        <v>3317.26089</v>
+        <v>2281.459959</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>2.265766</v>
+        <v>3.00442</v>
       </c>
     </row>
     <row r="10">
@@ -1654,32 +1654,32 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>U01</t>
+          <t>U06</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>A01</t>
+          <t>B03</t>
         </is>
       </c>
       <c r="E10" s="4" t="n">
-        <v>0</v>
+        <v>1440.969393</v>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>S009→S002</t>
+          <t>S007</t>
         </is>
       </c>
       <c r="G10" s="4" t="n">
-        <v>2281.459959</v>
+        <v>3062.28364</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>3.00442</v>
+        <v>1.773846</v>
       </c>
     </row>
     <row r="11">
@@ -1690,32 +1690,32 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>U02</t>
+          <t>U05</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>A02</t>
+          <t>B04</t>
         </is>
       </c>
       <c r="E11" s="4" t="n">
-        <v>0</v>
+        <v>1554.571359</v>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>S007</t>
+          <t>S014</t>
         </is>
       </c>
       <c r="G11" s="4" t="n">
-        <v>1712.441636</v>
+        <v>3399.110249</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>1.899072</v>
+        <v>2.127681</v>
       </c>
     </row>
     <row r="12">
@@ -1726,32 +1726,32 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>U06</t>
+          <t>U07</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>B04</t>
+          <t>C04</t>
         </is>
       </c>
       <c r="E12" s="4" t="n">
-        <v>1440.969393</v>
+        <v>2115.081641</v>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>S014→S010</t>
+          <t>S001</t>
         </is>
       </c>
       <c r="G12" s="4" t="n">
-        <v>3548.250366</v>
+        <v>3610.507819</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>2.322729</v>
+        <v>2.672703</v>
       </c>
     </row>
     <row r="13">
@@ -1762,32 +1762,32 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>U03</t>
+          <t>U07</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>A03</t>
+          <t>C02</t>
         </is>
       </c>
       <c r="E13" s="4" t="n">
-        <v>0</v>
+        <v>3610.507819</v>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>S012</t>
+          <t>S004</t>
         </is>
       </c>
       <c r="G13" s="4" t="n">
-        <v>2130.639089</v>
+        <v>5915.691884</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>2.969256</v>
+        <v>6.176911</v>
       </c>
     </row>
     <row r="14">
@@ -1798,32 +1798,32 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>U04</t>
+          <t>U06</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>A04</t>
+          <t>B01</t>
         </is>
       </c>
       <c r="E14" s="4" t="n">
-        <v>0</v>
+        <v>3062.28364</v>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>S001</t>
+          <t>S008</t>
         </is>
       </c>
       <c r="G14" s="4" t="n">
-        <v>1312.470877</v>
+        <v>5020.324912</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>1.268023</v>
+        <v>2.982875</v>
       </c>
     </row>
     <row r="15">
@@ -1834,7 +1834,7 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>U07</t>
+          <t>U08</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
@@ -1848,18 +1848,18 @@
         </is>
       </c>
       <c r="E15" s="4" t="n">
-        <v>4398.672189</v>
+        <v>4607.747359</v>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>S004</t>
+          <t>S003</t>
         </is>
       </c>
       <c r="G15" s="4" t="n">
-        <v>6571.856254</v>
+        <v>7043.55688</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>5.540004</v>
+        <v>6.14777</v>
       </c>
     </row>
     <row r="16">
@@ -1870,32 +1870,32 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>U05</t>
+          <t>U04</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>B01</t>
+          <t>A04</t>
         </is>
       </c>
       <c r="E16" s="4" t="n">
-        <v>3317.26089</v>
+        <v>0</v>
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>S008</t>
+          <t>S015→S003</t>
         </is>
       </c>
       <c r="G16" s="4" t="n">
-        <v>5275.302162</v>
+        <v>2608.040897</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>2.982875</v>
+        <v>3.16972</v>
       </c>
     </row>
     <row r="17">
@@ -1906,32 +1906,32 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>U06</t>
+          <t>U02</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>B02</t>
+          <t>A05</t>
         </is>
       </c>
       <c r="E17" s="4" t="n">
-        <v>3548.250366</v>
+        <v>1223.535214</v>
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>S008</t>
+          <t>S012</t>
         </is>
       </c>
       <c r="G17" s="4" t="n">
-        <v>5446.291637</v>
+        <v>3354.174302</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>2.77042</v>
+        <v>2.969256</v>
       </c>
     </row>
     <row r="18">
@@ -1942,7 +1942,7 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>U04</t>
+          <t>U01</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
@@ -1952,7 +1952,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>A05</t>
+          <t>A06</t>
         </is>
       </c>
       <c r="E18" s="4" t="n">
@@ -1960,14 +1960,14 @@
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>S004</t>
+          <t>S005</t>
         </is>
       </c>
       <c r="G18" s="4" t="n">
-        <v>3496.430278</v>
+        <v>3008.228982</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>3.098647</v>
+        <v>2.129519</v>
       </c>
     </row>
     <row r="19">
@@ -1978,32 +1978,32 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>U02</t>
+          <t>U05</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>A06</t>
+          <t>B02</t>
         </is>
       </c>
       <c r="E19" s="4" t="n">
-        <v>1712.441636</v>
+        <v>3399.110249</v>
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>S003→S015</t>
+          <t>S015→S003</t>
         </is>
       </c>
       <c r="G19" s="4" t="n">
-        <v>4260.482533</v>
+        <v>5682.242356</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>3.089952</v>
+        <v>3.0883</v>
       </c>
     </row>
     <row r="20">
@@ -2024,22 +2024,22 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>A04</t>
+          <t>A01</t>
         </is>
       </c>
       <c r="E20" s="4" t="n">
-        <v>2178.788712</v>
+        <v>2281.459959</v>
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>S011</t>
+          <t>S013→S012</t>
         </is>
       </c>
       <c r="G20" s="4" t="n">
-        <v>3402.323926</v>
+        <v>4625.307034</v>
       </c>
       <c r="H20" s="4" t="n">
-        <v>1.15549</v>
+        <v>2.98926</v>
       </c>
     </row>
     <row r="21">
@@ -2050,7 +2050,7 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>U05</t>
+          <t>U06</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
@@ -2064,18 +2064,18 @@
         </is>
       </c>
       <c r="E21" s="4" t="n">
-        <v>5275.302162</v>
+        <v>5020.324912</v>
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>S015→S003</t>
+          <t>S008</t>
         </is>
       </c>
       <c r="G21" s="4" t="n">
-        <v>7558.434268</v>
+        <v>6918.366183</v>
       </c>
       <c r="H21" s="4" t="n">
-        <v>3.0883</v>
+        <v>2.77042</v>
       </c>
     </row>
     <row r="22">
@@ -2086,7 +2086,7 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>U01</t>
+          <t>U04</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
@@ -2100,18 +2100,18 @@
         </is>
       </c>
       <c r="E22" s="4" t="n">
-        <v>2761.062337</v>
+        <v>2608.040897</v>
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>S005</t>
+          <t>S009</t>
         </is>
       </c>
       <c r="G22" s="4" t="n">
-        <v>4456.820442</v>
+        <v>4299.575383</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>2.129519</v>
+        <v>2.33825</v>
       </c>
     </row>
     <row r="23">
@@ -2122,248 +2122,32 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>U03</t>
+          <t>U07</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>A03</t>
+          <t>C04</t>
         </is>
       </c>
       <c r="E23" s="4" t="n">
-        <v>3488.424084</v>
+        <v>5915.691884</v>
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>S013→S012</t>
+          <t>S011→S005</t>
         </is>
       </c>
       <c r="G23" s="4" t="n">
-        <v>5832.271158</v>
+        <v>8027.342267</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>2.98926</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="4" t="inlineStr">
-        <is>
-          <t>T023</t>
-        </is>
-      </c>
-      <c r="B24" s="4" t="inlineStr">
-        <is>
-          <t>U04</t>
-        </is>
-      </c>
-      <c r="C24" s="4" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D24" s="4" t="inlineStr">
-        <is>
-          <t>A01</t>
-        </is>
-      </c>
-      <c r="E24" s="4" t="n">
-        <v>3649.403581</v>
-      </c>
-      <c r="F24" s="4" t="inlineStr">
-        <is>
-          <t>S005</t>
-        </is>
-      </c>
-      <c r="G24" s="4" t="n">
-        <v>5345.161685</v>
-      </c>
-      <c r="H24" s="4" t="n">
-        <v>2.201456</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="4" t="inlineStr">
-        <is>
-          <t>T024</t>
-        </is>
-      </c>
-      <c r="B25" s="4" t="inlineStr">
-        <is>
-          <t>U06</t>
-        </is>
-      </c>
-      <c r="C25" s="4" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D25" s="4" t="inlineStr">
-        <is>
-          <t>B04</t>
-        </is>
-      </c>
-      <c r="E25" s="4" t="n">
-        <v>5446.291637</v>
-      </c>
-      <c r="F25" s="4" t="inlineStr">
-        <is>
-          <t>S005</t>
-        </is>
-      </c>
-      <c r="G25" s="4" t="n">
-        <v>6965.315981</v>
-      </c>
-      <c r="H25" s="4" t="n">
-        <v>1.841574</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="4" t="inlineStr">
-        <is>
-          <t>T025</t>
-        </is>
-      </c>
-      <c r="B26" s="4" t="inlineStr">
-        <is>
-          <t>U02</t>
-        </is>
-      </c>
-      <c r="C26" s="4" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D26" s="4" t="inlineStr">
-        <is>
-          <t>A04</t>
-        </is>
-      </c>
-      <c r="E26" s="4" t="n">
-        <v>4260.482533</v>
-      </c>
-      <c r="F26" s="4" t="inlineStr">
-        <is>
-          <t>S009</t>
-        </is>
-      </c>
-      <c r="G26" s="4" t="n">
-        <v>5892.017019</v>
-      </c>
-      <c r="H26" s="4" t="n">
-        <v>2.22377</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="4" t="inlineStr">
-        <is>
-          <t>T026</t>
-        </is>
-      </c>
-      <c r="B27" s="4" t="inlineStr">
-        <is>
-          <t>U01</t>
-        </is>
-      </c>
-      <c r="C27" s="4" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D27" s="4" t="inlineStr">
-        <is>
-          <t>A05</t>
-        </is>
-      </c>
-      <c r="E27" s="4" t="n">
-        <v>4891.59501</v>
-      </c>
-      <c r="F27" s="4" t="inlineStr">
-        <is>
-          <t>S015</t>
-        </is>
-      </c>
-      <c r="G27" s="4" t="n">
-        <v>6801.804857</v>
-      </c>
-      <c r="H27" s="4" t="n">
-        <v>2.364455</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="4" t="inlineStr">
-        <is>
-          <t>T027</t>
-        </is>
-      </c>
-      <c r="B28" s="4" t="inlineStr">
-        <is>
-          <t>U04</t>
-        </is>
-      </c>
-      <c r="C28" s="4" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D28" s="4" t="inlineStr">
-        <is>
-          <t>A02</t>
-        </is>
-      </c>
-      <c r="E28" s="4" t="n">
-        <v>5572.014767</v>
-      </c>
-      <c r="F28" s="4" t="inlineStr">
-        <is>
-          <t>S009</t>
-        </is>
-      </c>
-      <c r="G28" s="4" t="n">
-        <v>7203.549253</v>
-      </c>
-      <c r="H28" s="4" t="n">
-        <v>2.164473</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="4" t="inlineStr">
-        <is>
-          <t>T028</t>
-        </is>
-      </c>
-      <c r="B29" s="4" t="inlineStr">
-        <is>
-          <t>U03</t>
-        </is>
-      </c>
-      <c r="C29" s="4" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D29" s="4" t="inlineStr">
-        <is>
-          <t>A06</t>
-        </is>
-      </c>
-      <c r="E29" s="4" t="n">
-        <v>5832.271158</v>
-      </c>
-      <c r="F29" s="4" t="inlineStr">
-        <is>
-          <t>S011</t>
-        </is>
-      </c>
-      <c r="G29" s="4" t="n">
-        <v>6995.806372</v>
-      </c>
-      <c r="H29" s="4" t="n">
-        <v>1.104775</v>
+        <v>4.069881</v>
       </c>
     </row>
   </sheetData>
@@ -2476,7 +2260,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>T006</t>
+          <t>T011</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
@@ -2485,7 +2269,7 @@
         </is>
       </c>
       <c r="D5" s="4" t="n">
-        <v>3587.495972</v>
+        <v>3297.97973</v>
       </c>
     </row>
     <row r="6">
@@ -2496,7 +2280,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>T006</t>
+          <t>T011</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
@@ -2505,7 +2289,7 @@
         </is>
       </c>
       <c r="D6" s="4" t="n">
-        <v>3587.495972</v>
+        <v>3297.97973</v>
       </c>
     </row>
     <row r="7">
@@ -2516,7 +2300,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>T013</t>
+          <t>T005</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -2536,7 +2320,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>T013</t>
+          <t>T005</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -2556,7 +2340,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>T013</t>
+          <t>T005</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
@@ -2576,7 +2360,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>T006</t>
+          <t>T011</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
@@ -2585,7 +2369,7 @@
         </is>
       </c>
       <c r="D10" s="4" t="n">
-        <v>3587.495972</v>
+        <v>3297.97973</v>
       </c>
     </row>
     <row r="11">
@@ -2596,7 +2380,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>T006</t>
+          <t>T011</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
@@ -2605,7 +2389,7 @@
         </is>
       </c>
       <c r="D11" s="4" t="n">
-        <v>3587.495972</v>
+        <v>3297.97973</v>
       </c>
     </row>
     <row r="12">
@@ -2616,7 +2400,7 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>T006</t>
+          <t>T011</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
@@ -2625,7 +2409,7 @@
         </is>
       </c>
       <c r="D12" s="4" t="n">
-        <v>3587.495972</v>
+        <v>3297.97973</v>
       </c>
     </row>
     <row r="13">
@@ -2636,7 +2420,7 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>T006</t>
+          <t>T011</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
@@ -2645,7 +2429,7 @@
         </is>
       </c>
       <c r="D13" s="4" t="n">
-        <v>3587.495972</v>
+        <v>3297.97973</v>
       </c>
     </row>
     <row r="14">
@@ -2716,7 +2500,7 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>T003</t>
+          <t>T001</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
@@ -2725,7 +2509,7 @@
         </is>
       </c>
       <c r="D17" s="4" t="n">
-        <v>2986.376998</v>
+        <v>1490.950821</v>
       </c>
     </row>
     <row r="18">
@@ -2736,7 +2520,7 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>T003</t>
+          <t>T001</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
@@ -2745,7 +2529,7 @@
         </is>
       </c>
       <c r="D18" s="4" t="n">
-        <v>2986.376998</v>
+        <v>1490.950821</v>
       </c>
     </row>
     <row r="19">
@@ -2756,7 +2540,7 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>T003</t>
+          <t>T001</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
@@ -2765,7 +2549,7 @@
         </is>
       </c>
       <c r="D19" s="4" t="n">
-        <v>2986.376998</v>
+        <v>1490.950821</v>
       </c>
     </row>
     <row r="20">
@@ -2776,7 +2560,7 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>T009</t>
+          <t>T008</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
@@ -2796,7 +2580,7 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>T009</t>
+          <t>T008</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
@@ -2816,7 +2600,7 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>T003</t>
+          <t>T001</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
@@ -2825,7 +2609,7 @@
         </is>
       </c>
       <c r="D22" s="4" t="n">
-        <v>2986.376998</v>
+        <v>1490.950821</v>
       </c>
     </row>
     <row r="23">
@@ -2836,7 +2620,7 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>T003</t>
+          <t>T001</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
@@ -2845,7 +2629,7 @@
         </is>
       </c>
       <c r="D23" s="4" t="n">
-        <v>2986.376998</v>
+        <v>1490.950821</v>
       </c>
     </row>
     <row r="24">
@@ -2856,7 +2640,7 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>T003</t>
+          <t>T001</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
@@ -2865,7 +2649,7 @@
         </is>
       </c>
       <c r="D24" s="4" t="n">
-        <v>2986.376998</v>
+        <v>1490.950821</v>
       </c>
     </row>
     <row r="25">
@@ -2876,7 +2660,7 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>T007</t>
+          <t>T014</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
@@ -2885,7 +2669,7 @@
         </is>
       </c>
       <c r="D25" s="4" t="n">
-        <v>5255.872579</v>
+        <v>6253.112119</v>
       </c>
     </row>
     <row r="26">
@@ -2896,7 +2680,7 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>T007</t>
+          <t>T014</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
@@ -2905,7 +2689,7 @@
         </is>
       </c>
       <c r="D26" s="4" t="n">
-        <v>5255.872579</v>
+        <v>6253.112119</v>
       </c>
     </row>
     <row r="27">
@@ -2916,7 +2700,7 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>T007</t>
+          <t>T014</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
@@ -2925,7 +2709,7 @@
         </is>
       </c>
       <c r="D27" s="4" t="n">
-        <v>5255.872579</v>
+        <v>6253.112119</v>
       </c>
     </row>
     <row r="28">
@@ -2936,7 +2720,7 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>T018</t>
+          <t>T015</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
@@ -2945,7 +2729,7 @@
         </is>
       </c>
       <c r="D28" s="4" t="n">
-        <v>3091.553465</v>
+        <v>1754.875734</v>
       </c>
     </row>
     <row r="29">
@@ -2956,7 +2740,7 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>T020</t>
+          <t>T018</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
@@ -2965,7 +2749,7 @@
         </is>
       </c>
       <c r="D29" s="4" t="n">
-        <v>6826.286864</v>
+        <v>4950.094952</v>
       </c>
     </row>
     <row r="30">
@@ -2976,7 +2760,7 @@
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>T007</t>
+          <t>T014</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
@@ -2985,7 +2769,7 @@
         </is>
       </c>
       <c r="D30" s="4" t="n">
-        <v>5255.872579</v>
+        <v>6253.112119</v>
       </c>
     </row>
     <row r="31">
@@ -2996,7 +2780,7 @@
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>T007</t>
+          <t>T014</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
@@ -3005,7 +2789,7 @@
         </is>
       </c>
       <c r="D31" s="4" t="n">
-        <v>5255.872579</v>
+        <v>6253.112119</v>
       </c>
     </row>
     <row r="32">
@@ -3016,7 +2800,7 @@
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>T007</t>
+          <t>T014</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
@@ -3025,7 +2809,7 @@
         </is>
       </c>
       <c r="D32" s="4" t="n">
-        <v>5255.872579</v>
+        <v>6253.112119</v>
       </c>
     </row>
     <row r="33">
@@ -3036,7 +2820,7 @@
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>T014</t>
+          <t>T012</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
@@ -3045,7 +2829,7 @@
         </is>
       </c>
       <c r="D33" s="4" t="n">
-        <v>5852.234222</v>
+        <v>5196.069851</v>
       </c>
     </row>
     <row r="34">
@@ -3056,7 +2840,7 @@
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>T014</t>
+          <t>T012</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
@@ -3065,7 +2849,7 @@
         </is>
       </c>
       <c r="D34" s="4" t="n">
-        <v>5852.234222</v>
+        <v>5196.069851</v>
       </c>
     </row>
     <row r="35">
@@ -3076,7 +2860,7 @@
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>T017</t>
+          <t>T012</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
@@ -3085,7 +2869,7 @@
         </is>
       </c>
       <c r="D35" s="4" t="n">
-        <v>2686.097244</v>
+        <v>5196.069851</v>
       </c>
     </row>
     <row r="36">
@@ -3096,7 +2880,7 @@
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>T017</t>
+          <t>T012</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
@@ -3105,7 +2889,7 @@
         </is>
       </c>
       <c r="D36" s="4" t="n">
-        <v>2686.097244</v>
+        <v>5196.069851</v>
       </c>
     </row>
     <row r="37">
@@ -3116,7 +2900,7 @@
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>T014</t>
+          <t>T012</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
@@ -3125,7 +2909,7 @@
         </is>
       </c>
       <c r="D37" s="4" t="n">
-        <v>5852.234222</v>
+        <v>5196.069851</v>
       </c>
     </row>
     <row r="38">
@@ -3136,7 +2920,7 @@
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>T014</t>
+          <t>T012</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
@@ -3145,7 +2929,7 @@
         </is>
       </c>
       <c r="D38" s="4" t="n">
-        <v>5852.234222</v>
+        <v>5196.069851</v>
       </c>
     </row>
     <row r="39">
@@ -3156,7 +2940,7 @@
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>T023</t>
+          <t>T022</t>
         </is>
       </c>
       <c r="C39" s="4" t="inlineStr">
@@ -3165,7 +2949,7 @@
         </is>
       </c>
       <c r="D39" s="4" t="n">
-        <v>4780.0393</v>
+        <v>7521.954947</v>
       </c>
     </row>
     <row r="40">
@@ -3176,7 +2960,7 @@
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>T024</t>
+          <t>T022</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
@@ -3185,7 +2969,7 @@
         </is>
       </c>
       <c r="D40" s="4" t="n">
-        <v>6488.560476</v>
+        <v>7521.954947</v>
       </c>
     </row>
     <row r="41">
@@ -3196,7 +2980,7 @@
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>T021</t>
+          <t>T017</t>
         </is>
       </c>
       <c r="C41" s="4" t="inlineStr">
@@ -3205,7 +2989,7 @@
         </is>
       </c>
       <c r="D41" s="4" t="n">
-        <v>3891.698056</v>
+        <v>2443.106596</v>
       </c>
     </row>
     <row r="42">
@@ -3216,7 +3000,7 @@
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>T021</t>
+          <t>T017</t>
         </is>
       </c>
       <c r="C42" s="4" t="inlineStr">
@@ -3225,7 +3009,7 @@
         </is>
       </c>
       <c r="D42" s="4" t="n">
-        <v>3891.698056</v>
+        <v>2443.106596</v>
       </c>
     </row>
     <row r="43">
@@ -3236,7 +3020,7 @@
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>T023</t>
+          <t>T022</t>
         </is>
       </c>
       <c r="C43" s="4" t="inlineStr">
@@ -3245,7 +3029,7 @@
         </is>
       </c>
       <c r="D43" s="4" t="n">
-        <v>4780.0393</v>
+        <v>7521.954947</v>
       </c>
     </row>
     <row r="44">
@@ -3256,7 +3040,7 @@
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>T024</t>
+          <t>T022</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
@@ -3265,7 +3049,7 @@
         </is>
       </c>
       <c r="D44" s="4" t="n">
-        <v>6488.560476</v>
+        <v>7521.954947</v>
       </c>
     </row>
     <row r="45">
@@ -3276,7 +3060,7 @@
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>T001</t>
+          <t>T007</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
@@ -3285,7 +3069,7 @@
         </is>
       </c>
       <c r="D45" s="4" t="n">
-        <v>1169.162541</v>
+        <v>2766.588719</v>
       </c>
     </row>
     <row r="46">
@@ -3296,7 +3080,7 @@
       </c>
       <c r="B46" s="4" t="inlineStr">
         <is>
-          <t>T001</t>
+          <t>T007</t>
         </is>
       </c>
       <c r="C46" s="4" t="inlineStr">
@@ -3305,7 +3089,7 @@
         </is>
       </c>
       <c r="D46" s="4" t="n">
-        <v>1169.162541</v>
+        <v>2766.588719</v>
       </c>
     </row>
     <row r="47">
@@ -3316,7 +3100,7 @@
       </c>
       <c r="B47" s="4" t="inlineStr">
         <is>
-          <t>T004</t>
+          <t>T007</t>
         </is>
       </c>
       <c r="C47" s="4" t="inlineStr">
@@ -3325,7 +3109,7 @@
         </is>
       </c>
       <c r="D47" s="4" t="n">
-        <v>883.753292</v>
+        <v>2766.588719</v>
       </c>
     </row>
     <row r="48">
@@ -3336,7 +3120,7 @@
       </c>
       <c r="B48" s="4" t="inlineStr">
         <is>
-          <t>T004</t>
+          <t>T007</t>
         </is>
       </c>
       <c r="C48" s="4" t="inlineStr">
@@ -3345,7 +3129,7 @@
         </is>
       </c>
       <c r="D48" s="4" t="n">
-        <v>883.753292</v>
+        <v>2766.588719</v>
       </c>
     </row>
     <row r="49">
@@ -3356,7 +3140,7 @@
       </c>
       <c r="B49" s="4" t="inlineStr">
         <is>
-          <t>T001</t>
+          <t>T007</t>
         </is>
       </c>
       <c r="C49" s="4" t="inlineStr">
@@ -3365,7 +3149,7 @@
         </is>
       </c>
       <c r="D49" s="4" t="n">
-        <v>1169.162541</v>
+        <v>2766.588719</v>
       </c>
     </row>
     <row r="50">
@@ -3376,7 +3160,7 @@
       </c>
       <c r="B50" s="4" t="inlineStr">
         <is>
-          <t>T001</t>
+          <t>T007</t>
         </is>
       </c>
       <c r="C50" s="4" t="inlineStr">
@@ -3385,7 +3169,7 @@
         </is>
       </c>
       <c r="D50" s="4" t="n">
-        <v>1169.162541</v>
+        <v>2766.588719</v>
       </c>
     </row>
     <row r="51">
@@ -3396,7 +3180,7 @@
       </c>
       <c r="B51" s="4" t="inlineStr">
         <is>
-          <t>T001</t>
+          <t>T009</t>
         </is>
       </c>
       <c r="C51" s="4" t="inlineStr">
@@ -3405,7 +3189,7 @@
         </is>
       </c>
       <c r="D51" s="4" t="n">
-        <v>1853.94568</v>
+        <v>2559.266516</v>
       </c>
     </row>
     <row r="52">
@@ -3416,7 +3200,7 @@
       </c>
       <c r="B52" s="4" t="inlineStr">
         <is>
-          <t>T001</t>
+          <t>T007</t>
         </is>
       </c>
       <c r="C52" s="4" t="inlineStr">
@@ -3425,7 +3209,7 @@
         </is>
       </c>
       <c r="D52" s="4" t="n">
-        <v>1853.94568</v>
+        <v>3415.371857</v>
       </c>
     </row>
     <row r="53">
@@ -3436,7 +3220,7 @@
       </c>
       <c r="B53" s="4" t="inlineStr">
         <is>
-          <t>T010</t>
+          <t>T009</t>
         </is>
       </c>
       <c r="C53" s="4" t="inlineStr">
@@ -3445,7 +3229,7 @@
         </is>
       </c>
       <c r="D53" s="4" t="n">
-        <v>1133.860818</v>
+        <v>2559.266516</v>
       </c>
     </row>
     <row r="54">
@@ -3456,7 +3240,7 @@
       </c>
       <c r="B54" s="4" t="inlineStr">
         <is>
-          <t>T010</t>
+          <t>T009</t>
         </is>
       </c>
       <c r="C54" s="4" t="inlineStr">
@@ -3465,7 +3249,7 @@
         </is>
       </c>
       <c r="D54" s="4" t="n">
-        <v>1133.860818</v>
+        <v>2559.266516</v>
       </c>
     </row>
     <row r="55">
@@ -3476,7 +3260,7 @@
       </c>
       <c r="B55" s="4" t="inlineStr">
         <is>
-          <t>T001</t>
+          <t>T007</t>
         </is>
       </c>
       <c r="C55" s="4" t="inlineStr">
@@ -3485,7 +3269,7 @@
         </is>
       </c>
       <c r="D55" s="4" t="n">
-        <v>1853.94568</v>
+        <v>3415.371857</v>
       </c>
     </row>
     <row r="56">
@@ -3496,7 +3280,7 @@
       </c>
       <c r="B56" s="4" t="inlineStr">
         <is>
-          <t>T015</t>
+          <t>T013</t>
         </is>
       </c>
       <c r="C56" s="4" t="inlineStr">
@@ -3505,7 +3289,7 @@
         </is>
       </c>
       <c r="D56" s="4" t="n">
-        <v>4606.508193</v>
+        <v>4351.530943</v>
       </c>
     </row>
     <row r="57">
@@ -3516,7 +3300,7 @@
       </c>
       <c r="B57" s="4" t="inlineStr">
         <is>
-          <t>T016</t>
+          <t>T020</t>
         </is>
       </c>
       <c r="C57" s="4" t="inlineStr">
@@ -3525,7 +3309,7 @@
         </is>
       </c>
       <c r="D57" s="4" t="n">
-        <v>4777.497668</v>
+        <v>6249.572214</v>
       </c>
     </row>
     <row r="58">
@@ -3536,7 +3320,7 @@
       </c>
       <c r="B58" s="4" t="inlineStr">
         <is>
-          <t>T015</t>
+          <t>T013</t>
         </is>
       </c>
       <c r="C58" s="4" t="inlineStr">
@@ -3545,7 +3329,7 @@
         </is>
       </c>
       <c r="D58" s="4" t="n">
-        <v>4606.508193</v>
+        <v>4351.530943</v>
       </c>
     </row>
     <row r="59">
@@ -3556,7 +3340,7 @@
       </c>
       <c r="B59" s="4" t="inlineStr">
         <is>
-          <t>T015</t>
+          <t>T013</t>
         </is>
       </c>
       <c r="C59" s="4" t="inlineStr">
@@ -3565,7 +3349,7 @@
         </is>
       </c>
       <c r="D59" s="4" t="n">
-        <v>4606.508193</v>
+        <v>4351.530943</v>
       </c>
     </row>
     <row r="60">
@@ -3576,7 +3360,7 @@
       </c>
       <c r="B60" s="4" t="inlineStr">
         <is>
-          <t>T016</t>
+          <t>T020</t>
         </is>
       </c>
       <c r="C60" s="4" t="inlineStr">
@@ -3585,7 +3369,7 @@
         </is>
       </c>
       <c r="D60" s="4" t="n">
-        <v>4777.497668</v>
+        <v>6249.572214</v>
       </c>
     </row>
     <row r="61">
@@ -3596,7 +3380,7 @@
       </c>
       <c r="B61" s="4" t="inlineStr">
         <is>
-          <t>T027</t>
+          <t>T021</t>
         </is>
       </c>
       <c r="C61" s="4" t="inlineStr">
@@ -3605,7 +3389,7 @@
         </is>
       </c>
       <c r="D61" s="4" t="n">
-        <v>6639.37201</v>
+        <v>3735.39814</v>
       </c>
     </row>
     <row r="62">
@@ -3616,7 +3400,7 @@
       </c>
       <c r="B62" s="4" t="inlineStr">
         <is>
-          <t>T009</t>
+          <t>T008</t>
         </is>
       </c>
       <c r="C62" s="4" t="inlineStr">
@@ -3636,7 +3420,7 @@
       </c>
       <c r="B63" s="4" t="inlineStr">
         <is>
-          <t>T025</t>
+          <t>T021</t>
         </is>
       </c>
       <c r="C63" s="4" t="inlineStr">
@@ -3645,7 +3429,7 @@
         </is>
       </c>
       <c r="D63" s="4" t="n">
-        <v>5327.839776</v>
+        <v>3735.39814</v>
       </c>
     </row>
     <row r="64">
@@ -3656,7 +3440,7 @@
       </c>
       <c r="B64" s="4" t="inlineStr">
         <is>
-          <t>T011</t>
+          <t>T003</t>
         </is>
       </c>
       <c r="C64" s="4" t="inlineStr">
@@ -3665,7 +3449,7 @@
         </is>
       </c>
       <c r="D64" s="4" t="n">
-        <v>3078.501353</v>
+        <v>1084.822346</v>
       </c>
     </row>
     <row r="65">
@@ -3676,7 +3460,7 @@
       </c>
       <c r="B65" s="4" t="inlineStr">
         <is>
-          <t>T008</t>
+          <t>T003</t>
         </is>
       </c>
       <c r="C65" s="4" t="inlineStr">
@@ -3685,7 +3469,7 @@
         </is>
       </c>
       <c r="D65" s="4" t="n">
-        <v>2264.802263</v>
+        <v>1084.822346</v>
       </c>
     </row>
     <row r="66">
@@ -3696,7 +3480,7 @@
       </c>
       <c r="B66" s="4" t="inlineStr">
         <is>
-          <t>T008</t>
+          <t>T003</t>
         </is>
       </c>
       <c r="C66" s="4" t="inlineStr">
@@ -3705,7 +3489,7 @@
         </is>
       </c>
       <c r="D66" s="4" t="n">
-        <v>2264.802263</v>
+        <v>1084.822346</v>
       </c>
     </row>
     <row r="67">
@@ -3716,7 +3500,7 @@
       </c>
       <c r="B67" s="4" t="inlineStr">
         <is>
-          <t>T028</t>
+          <t>T022</t>
         </is>
       </c>
       <c r="C67" s="4" t="inlineStr">
@@ -3725,7 +3509,7 @@
         </is>
       </c>
       <c r="D67" s="4" t="n">
-        <v>6666.225432</v>
+        <v>6878.197319</v>
       </c>
     </row>
     <row r="68">
@@ -3736,7 +3520,7 @@
       </c>
       <c r="B68" s="4" t="inlineStr">
         <is>
-          <t>T019</t>
+          <t>T006</t>
         </is>
       </c>
       <c r="C68" s="4" t="inlineStr">
@@ -3745,7 +3529,7 @@
         </is>
       </c>
       <c r="D68" s="4" t="n">
-        <v>3072.742986</v>
+        <v>893.9542729999999</v>
       </c>
     </row>
     <row r="69">
@@ -3756,7 +3540,7 @@
       </c>
       <c r="B69" s="4" t="inlineStr">
         <is>
-          <t>T019</t>
+          <t>T006</t>
         </is>
       </c>
       <c r="C69" s="4" t="inlineStr">
@@ -3765,7 +3549,7 @@
         </is>
       </c>
       <c r="D69" s="4" t="n">
-        <v>3072.742986</v>
+        <v>893.9542729999999</v>
       </c>
     </row>
     <row r="70">
@@ -3776,7 +3560,7 @@
       </c>
       <c r="B70" s="4" t="inlineStr">
         <is>
-          <t>T022</t>
+          <t>T019</t>
         </is>
       </c>
       <c r="C70" s="4" t="inlineStr">
@@ -3785,7 +3569,7 @@
         </is>
       </c>
       <c r="D70" s="4" t="n">
-        <v>5046.881614</v>
+        <v>3839.917489</v>
       </c>
     </row>
     <row r="71">
@@ -3796,7 +3580,7 @@
       </c>
       <c r="B71" s="4" t="inlineStr">
         <is>
-          <t>T012</t>
+          <t>T016</t>
         </is>
       </c>
       <c r="C71" s="4" t="inlineStr">
@@ -3805,7 +3589,7 @@
         </is>
       </c>
       <c r="D71" s="4" t="n">
-        <v>1345.249544</v>
+        <v>2568.784758</v>
       </c>
     </row>
     <row r="72">
@@ -3816,7 +3600,7 @@
       </c>
       <c r="B72" s="4" t="inlineStr">
         <is>
-          <t>T012</t>
+          <t>T016</t>
         </is>
       </c>
       <c r="C72" s="4" t="inlineStr">
@@ -3825,7 +3609,7 @@
         </is>
       </c>
       <c r="D72" s="4" t="n">
-        <v>1345.249544</v>
+        <v>2568.784758</v>
       </c>
     </row>
     <row r="73">
@@ -3836,7 +3620,7 @@
       </c>
       <c r="B73" s="4" t="inlineStr">
         <is>
-          <t>T022</t>
+          <t>T019</t>
         </is>
       </c>
       <c r="C73" s="4" t="inlineStr">
@@ -3845,7 +3629,7 @@
         </is>
       </c>
       <c r="D73" s="4" t="n">
-        <v>4537.253785</v>
+        <v>3330.28966</v>
       </c>
     </row>
     <row r="74">
@@ -3856,7 +3640,7 @@
       </c>
       <c r="B74" s="4" t="inlineStr">
         <is>
-          <t>T005</t>
+          <t>T004</t>
         </is>
       </c>
       <c r="C74" s="4" t="inlineStr">
@@ -3876,7 +3660,7 @@
       </c>
       <c r="B75" s="4" t="inlineStr">
         <is>
-          <t>T005</t>
+          <t>T004</t>
         </is>
       </c>
       <c r="C75" s="4" t="inlineStr">
@@ -3896,7 +3680,7 @@
       </c>
       <c r="B76" s="4" t="inlineStr">
         <is>
-          <t>T008</t>
+          <t>T010</t>
         </is>
       </c>
       <c r="C76" s="4" t="inlineStr">
@@ -3905,7 +3689,7 @@
         </is>
       </c>
       <c r="D76" s="4" t="n">
-        <v>2702.548112</v>
+        <v>2784.397471</v>
       </c>
     </row>
     <row r="77">
@@ -3916,7 +3700,7 @@
       </c>
       <c r="B77" s="4" t="inlineStr">
         <is>
-          <t>T011</t>
+          <t>T010</t>
         </is>
       </c>
       <c r="C77" s="4" t="inlineStr">
@@ -3925,7 +3709,7 @@
         </is>
       </c>
       <c r="D77" s="4" t="n">
-        <v>2640.795504</v>
+        <v>2784.397471</v>
       </c>
     </row>
     <row r="78">
@@ -3936,7 +3720,7 @@
       </c>
       <c r="B78" s="4" t="inlineStr">
         <is>
-          <t>T011</t>
+          <t>T010</t>
         </is>
       </c>
       <c r="C78" s="4" t="inlineStr">
@@ -3945,7 +3729,7 @@
         </is>
       </c>
       <c r="D78" s="4" t="n">
-        <v>2640.795504</v>
+        <v>2784.397471</v>
       </c>
     </row>
     <row r="79">
@@ -3956,7 +3740,7 @@
       </c>
       <c r="B79" s="4" t="inlineStr">
         <is>
-          <t>T026</t>
+          <t>T015</t>
         </is>
       </c>
       <c r="C79" s="4" t="inlineStr">
@@ -3965,7 +3749,7 @@
         </is>
       </c>
       <c r="D79" s="4" t="n">
-        <v>6090.139933</v>
+        <v>1288.544923</v>
       </c>
     </row>
     <row r="80">
@@ -3976,7 +3760,7 @@
       </c>
       <c r="B80" s="4" t="inlineStr">
         <is>
-          <t>T018</t>
+          <t>T015</t>
         </is>
       </c>
       <c r="C80" s="4" t="inlineStr">
@@ -3985,7 +3769,7 @@
         </is>
       </c>
       <c r="D80" s="4" t="n">
-        <v>3548.817609</v>
+        <v>1288.544923</v>
       </c>
     </row>
     <row r="81">
@@ -3996,7 +3780,7 @@
       </c>
       <c r="B81" s="4" t="inlineStr">
         <is>
-          <t>T020</t>
+          <t>T018</t>
         </is>
       </c>
       <c r="C81" s="4" t="inlineStr">
@@ -4005,7 +3789,7 @@
         </is>
       </c>
       <c r="D81" s="4" t="n">
-        <v>6403.528658</v>
+        <v>4527.336746</v>
       </c>
     </row>
   </sheetData>

</xml_diff>